<commit_message>
save 09 09 2026
</commit_message>
<xml_diff>
--- a/4 четверть_26_Cursor.xlsx
+++ b/4 четверть_26_Cursor.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AlexServHW\Desktop\GB_Developer_Workbook\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{156DC75B-1E52-49B9-8524-BD442261E9F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DEB56677-167D-48E6-B1BB-7B968CDF378B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7635" yWindow="-18330" windowWidth="23250" windowHeight="12450" firstSheet="1" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-13875" yWindow="-21720" windowWidth="51840" windowHeight="21120" firstSheet="1" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Учебные матриалы" sheetId="7" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="659" uniqueCount="563">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="660" uniqueCount="564">
   <si>
     <t>Настройки Cursor</t>
   </si>
@@ -5360,17 +5360,60 @@
 AI:  Archived to openspec/changes/archive/2025-01-23-add-dark-mode/
      Specs updated. Ready for the next feature.</t>
   </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t># Скопировать папку pptx из репозитория</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+git clone https://github.com/anthropics/skills.git
+cp -r skills/skills/pptx ~/.cursor/skills/pptx</t>
+    </r>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="48" x14ac:knownFonts="1">
+  <fonts count="50" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -5822,9 +5865,9 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="39" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="88">
+  <cellXfs count="89">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top"/>
@@ -5832,13 +5875,13 @@
     <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="33" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="35" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="33" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="35" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
@@ -5848,7 +5891,7 @@
     <xf numFmtId="49" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="32" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="34" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
@@ -5861,90 +5904,120 @@
     <xf numFmtId="49" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="38" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="49" fontId="31" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="33" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="37" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="39" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="34" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="36" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="38" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="40" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="33" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="35" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="32" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="36" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="42" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="32" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="36" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="36" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="36" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="41" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="49" fontId="31" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="30" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="34" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="40" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="49" fontId="30" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="34" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="34" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="34" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="39" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="49" fontId="29" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="28" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="28" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="27" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="33" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="35" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="45" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="47" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="29" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="28" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="27" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="26" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="26" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="37" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="26" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="26" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="45" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="49" fontId="25" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="49" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="49" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="25" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
     </xf>
     <xf numFmtId="49" fontId="24" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -5952,58 +6025,31 @@
     <xf numFmtId="49" fontId="24" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="35" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="24" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="24" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="43" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="49" fontId="23" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="47" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="47" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="23" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
     </xf>
     <xf numFmtId="49" fontId="22" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="22" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="49" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="47" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
     </xf>
     <xf numFmtId="49" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="47" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="49" fontId="47" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
     <xf numFmtId="49" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="45" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
     <xf numFmtId="49" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="45" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="49" fontId="45" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
     </xf>
     <xf numFmtId="49" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -6023,20 +6069,20 @@
     <xf numFmtId="49" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
     <xf numFmtId="49" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="47" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
     <xf numFmtId="49" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="45" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -6044,21 +6090,21 @@
     <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="47" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="45" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -6071,7 +6117,7 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
+      <alignment vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -6153,9 +6199,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>2113177</xdr:colOff>
+      <xdr:colOff>2116987</xdr:colOff>
       <xdr:row>14</xdr:row>
-      <xdr:rowOff>1200835</xdr:rowOff>
+      <xdr:rowOff>1197025</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -9544,7 +9590,7 @@
       <c r="B10" s="21" t="s">
         <v>53</v>
       </c>
-      <c r="C10" s="64" t="s">
+      <c r="C10" s="63" t="s">
         <v>470</v>
       </c>
     </row>
@@ -9553,13 +9599,13 @@
       <c r="B11" s="21" t="s">
         <v>471</v>
       </c>
-      <c r="C11" s="64" t="s">
+      <c r="C11" s="63" t="s">
         <v>468</v>
       </c>
     </row>
     <row r="12" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A12" s="21"/>
-      <c r="C12" s="64"/>
+      <c r="C12" s="63"/>
     </row>
     <row r="13" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A13" s="2"/>
@@ -9643,7 +9689,7 @@
       <c r="B22" s="21" t="s">
         <v>272</v>
       </c>
-      <c r="C22" s="66" t="s">
+      <c r="C22" s="65" t="s">
         <v>273</v>
       </c>
     </row>
@@ -9691,7 +9737,7 @@
       </c>
     </row>
     <row r="28" spans="1:4" ht="331.2" x14ac:dyDescent="0.3">
-      <c r="B28" s="66" t="s">
+      <c r="B28" s="65" t="s">
         <v>475</v>
       </c>
       <c r="C28" s="21" t="s">
@@ -9856,7 +9902,7 @@
       <c r="B49" s="21" t="s">
         <v>483</v>
       </c>
-      <c r="C49" s="68" t="s">
+      <c r="C49" s="67" t="s">
         <v>438</v>
       </c>
     </row>
@@ -9881,12 +9927,15 @@
         <v>289</v>
       </c>
     </row>
-    <row r="53" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A53" s="22" t="s">
         <v>287</v>
       </c>
       <c r="B53" s="35" t="s">
         <v>288</v>
+      </c>
+      <c r="C53" s="87" t="s">
+        <v>563</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.3">
@@ -9902,7 +9951,7 @@
       <c r="B55" s="21" t="s">
         <v>482</v>
       </c>
-      <c r="C55" s="68" t="s">
+      <c r="C55" s="67" t="s">
         <v>484</v>
       </c>
     </row>
@@ -10483,7 +10532,7 @@
       <c r="B15" s="59" t="s">
         <v>442</v>
       </c>
-      <c r="C15" s="84" t="s">
+      <c r="C15" s="87" t="s">
         <v>441</v>
       </c>
     </row>
@@ -10534,7 +10583,7 @@
       <c r="C19" s="43" t="s">
         <v>406</v>
       </c>
-      <c r="D19" s="76" t="s">
+      <c r="D19" s="75" t="s">
         <v>404</v>
       </c>
     </row>
@@ -10548,7 +10597,7 @@
       <c r="C20" s="43" t="s">
         <v>408</v>
       </c>
-      <c r="D20" s="84" t="s">
+      <c r="D20" s="83" t="s">
         <v>407</v>
       </c>
     </row>
@@ -10562,7 +10611,7 @@
       <c r="C21" s="49" t="s">
         <v>420</v>
       </c>
-      <c r="D21" s="87" t="s">
+      <c r="D21" s="86" t="s">
         <v>418</v>
       </c>
     </row>
@@ -10610,23 +10659,23 @@
       <c r="D26" s="49"/>
     </row>
     <row r="27" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="B27" s="73" t="s">
+      <c r="B27" s="72" t="s">
         <v>501</v>
       </c>
       <c r="C27" s="49"/>
       <c r="D27" s="49"/>
     </row>
     <row r="28" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A28" s="74" t="s">
+      <c r="A28" s="73" t="s">
         <v>502</v>
       </c>
-      <c r="B28" s="73"/>
+      <c r="B28" s="72"/>
       <c r="C28" s="49"/>
       <c r="D28" s="49"/>
     </row>
     <row r="29" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="B29" s="73"/>
-      <c r="C29" s="75" t="s">
+      <c r="B29" s="72"/>
+      <c r="C29" s="74" t="s">
         <v>504</v>
       </c>
       <c r="D29" s="49"/>
@@ -10643,7 +10692,7 @@
       <c r="B31" s="1" t="s">
         <v>493</v>
       </c>
-      <c r="C31" s="75" t="s">
+      <c r="C31" s="74" t="s">
         <v>494</v>
       </c>
       <c r="D31" s="49"/>
@@ -10653,7 +10702,7 @@
         <v>495</v>
       </c>
       <c r="B32" s="1"/>
-      <c r="C32" s="73"/>
+      <c r="C32" s="72"/>
       <c r="D32" s="49"/>
     </row>
     <row r="33" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
@@ -10667,10 +10716,10 @@
       <c r="B34" s="21" t="s">
         <v>499</v>
       </c>
-      <c r="C34" s="85" t="s">
+      <c r="C34" s="84" t="s">
         <v>505</v>
       </c>
-      <c r="D34" s="73" t="s">
+      <c r="D34" s="72" t="s">
         <v>498</v>
       </c>
     </row>
@@ -10678,7 +10727,7 @@
       <c r="B35" s="21" t="s">
         <v>497</v>
       </c>
-      <c r="C35" s="73" t="s">
+      <c r="C35" s="72" t="s">
         <v>496</v>
       </c>
       <c r="D35" s="49"/>
@@ -10692,10 +10741,10 @@
       <c r="D36" s="49"/>
     </row>
     <row r="37" spans="1:4" ht="72" x14ac:dyDescent="0.3">
-      <c r="B37" s="70" t="s">
+      <c r="B37" s="69" t="s">
         <v>488</v>
       </c>
-      <c r="C37" s="77" t="s">
+      <c r="C37" s="76" t="s">
         <v>487</v>
       </c>
       <c r="D37" s="49"/>
@@ -10712,7 +10761,7 @@
       <c r="B39" s="1" t="s">
         <v>473</v>
       </c>
-      <c r="C39" s="65" t="s">
+      <c r="C39" s="64" t="s">
         <v>474</v>
       </c>
       <c r="D39" s="49"/>
@@ -10725,26 +10774,26 @@
       <c r="C40" s="43"/>
     </row>
     <row r="41" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="B41" s="71" t="s">
+      <c r="B41" s="70" t="s">
         <v>491</v>
       </c>
-      <c r="C41" s="71" t="s">
+      <c r="C41" s="70" t="s">
         <v>489</v>
       </c>
     </row>
     <row r="42" spans="1:4" ht="106.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B42" s="73" t="s">
+      <c r="B42" s="72" t="s">
         <v>503</v>
       </c>
-      <c r="C42" s="73" t="s">
+      <c r="C42" s="72" t="s">
         <v>504</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B43" s="72" t="s">
+      <c r="B43" s="71" t="s">
         <v>490</v>
       </c>
-      <c r="C43" s="63" t="s">
+      <c r="C43" s="88" t="s">
         <v>383</v>
       </c>
     </row>
@@ -10765,7 +10814,7 @@
       <c r="B46" s="21" t="s">
         <v>320</v>
       </c>
-      <c r="C46" s="69" t="s">
+      <c r="C46" s="68" t="s">
         <v>318</v>
       </c>
       <c r="D46" s="31" t="s">
@@ -10776,7 +10825,7 @@
       <c r="B47" s="21" t="s">
         <v>322</v>
       </c>
-      <c r="C47" s="84" t="s">
+      <c r="C47" s="83" t="s">
         <v>321</v>
       </c>
     </row>
@@ -11099,7 +11148,7 @@
       <c r="B84" s="21" t="s">
         <v>479</v>
       </c>
-      <c r="C84" s="67" t="s">
+      <c r="C84" s="66" t="s">
         <v>478</v>
       </c>
     </row>
@@ -11226,7 +11275,7 @@
     </row>
     <row r="10" spans="1:21" s="38" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B10" s="36"/>
-      <c r="C10" s="83" t="s">
+      <c r="C10" s="82" t="s">
         <v>536</v>
       </c>
       <c r="G10" s="36"/>
@@ -11239,7 +11288,7 @@
     </row>
     <row r="11" spans="1:21" s="38" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B11" s="36"/>
-      <c r="C11" s="82" t="s">
+      <c r="C11" s="81" t="s">
         <v>557</v>
       </c>
       <c r="G11" s="36"/>
@@ -11251,29 +11300,29 @@
       <c r="U11" s="36"/>
     </row>
     <row r="12" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A12" s="79" t="s">
+      <c r="A12" s="78" t="s">
         <v>506</v>
       </c>
       <c r="B12" s="49"/>
       <c r="C12" s="49"/>
-      <c r="D12" s="78"/>
+      <c r="D12" s="77"/>
     </row>
     <row r="13" spans="1:21" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="87" t="s">
+      <c r="A13" s="86" t="s">
         <v>507</v>
       </c>
       <c r="B13" s="49"/>
-      <c r="C13" s="78" t="s">
+      <c r="C13" s="77" t="s">
         <v>509</v>
       </c>
       <c r="D13" s="49"/>
     </row>
     <row r="14" spans="1:21" ht="72" x14ac:dyDescent="0.3">
-      <c r="A14" s="87" t="s">
+      <c r="A14" s="86" t="s">
         <v>508</v>
       </c>
       <c r="B14" s="49"/>
-      <c r="C14" s="78" t="s">
+      <c r="C14" s="77" t="s">
         <v>510</v>
       </c>
       <c r="D14" s="49"/>
@@ -11283,31 +11332,31 @@
         <v>515</v>
       </c>
       <c r="B15" s="49"/>
-      <c r="C15" s="78"/>
+      <c r="C15" s="77"/>
       <c r="D15" s="49"/>
     </row>
     <row r="16" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A16" s="78"/>
+      <c r="A16" s="77"/>
       <c r="B16" s="49"/>
-      <c r="C16" s="78" t="s">
+      <c r="C16" s="77" t="s">
         <v>516</v>
       </c>
       <c r="D16" s="49"/>
     </row>
     <row r="17" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="B17" s="78" t="s">
+      <c r="B17" s="77" t="s">
         <v>517</v>
       </c>
-      <c r="C17" s="78" t="s">
+      <c r="C17" s="77" t="s">
         <v>518</v>
       </c>
       <c r="D17" s="49"/>
     </row>
     <row r="18" spans="1:21" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="B18" s="78" t="s">
+      <c r="B18" s="77" t="s">
         <v>519</v>
       </c>
-      <c r="C18" s="78" t="s">
+      <c r="C18" s="77" t="s">
         <v>520</v>
       </c>
       <c r="D18" s="49"/>
@@ -11316,35 +11365,35 @@
       <c r="A19" s="11" t="s">
         <v>537</v>
       </c>
-      <c r="B19" s="78"/>
-      <c r="C19" s="78"/>
+      <c r="B19" s="77"/>
+      <c r="C19" s="77"/>
       <c r="D19" s="49"/>
     </row>
     <row r="20" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A20" s="80" t="s">
+      <c r="A20" s="79" t="s">
         <v>535</v>
       </c>
-      <c r="B20" s="78" t="s">
+      <c r="B20" s="77" t="s">
         <v>534</v>
       </c>
-      <c r="C20" s="78"/>
+      <c r="C20" s="77"/>
       <c r="D20" s="49"/>
     </row>
     <row r="21" spans="1:21" ht="100.8" x14ac:dyDescent="0.3">
-      <c r="A21" s="78"/>
-      <c r="B21" s="78"/>
-      <c r="C21" s="78" t="s">
+      <c r="A21" s="77"/>
+      <c r="B21" s="77"/>
+      <c r="C21" s="77" t="s">
         <v>543</v>
       </c>
-      <c r="D21" s="86" t="s">
+      <c r="D21" s="85" t="s">
         <v>559</v>
       </c>
     </row>
     <row r="22" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A22" s="80" t="s">
+      <c r="A22" s="79" t="s">
         <v>511</v>
       </c>
-      <c r="B22" s="78" t="s">
+      <c r="B22" s="77" t="s">
         <v>268</v>
       </c>
       <c r="C22" s="49"/>
@@ -11352,29 +11401,29 @@
     </row>
     <row r="23" spans="1:21" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A23" s="49"/>
-      <c r="B23" s="78" t="s">
+      <c r="B23" s="77" t="s">
         <v>513</v>
       </c>
-      <c r="C23" s="78" t="s">
+      <c r="C23" s="77" t="s">
         <v>512</v>
       </c>
-      <c r="D23" s="86" t="s">
+      <c r="D23" s="85" t="s">
         <v>560</v>
       </c>
     </row>
     <row r="24" spans="1:21" ht="72" x14ac:dyDescent="0.3">
       <c r="A24" s="49"/>
-      <c r="B24" s="78" t="s">
+      <c r="B24" s="77" t="s">
         <v>514</v>
       </c>
       <c r="C24" s="1"/>
       <c r="D24" s="49"/>
     </row>
     <row r="25" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A25" s="80" t="s">
+      <c r="A25" s="79" t="s">
         <v>521</v>
       </c>
-      <c r="B25" s="78" t="s">
+      <c r="B25" s="77" t="s">
         <v>269</v>
       </c>
       <c r="D25" s="49"/>
@@ -11382,7 +11431,7 @@
     <row r="26" spans="1:21" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A26" s="49"/>
       <c r="B26" s="49"/>
-      <c r="C26" s="78" t="s">
+      <c r="C26" s="77" t="s">
         <v>522</v>
       </c>
       <c r="D26" s="49"/>
@@ -11402,10 +11451,10 @@
       <c r="U26" s="21"/>
     </row>
     <row r="27" spans="1:21" s="6" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="80" t="s">
+      <c r="A27" s="79" t="s">
         <v>523</v>
       </c>
-      <c r="B27" s="78" t="s">
+      <c r="B27" s="77" t="s">
         <v>271</v>
       </c>
       <c r="C27" s="49"/>
@@ -11428,10 +11477,10 @@
     <row r="28" spans="1:21" s="6" customFormat="1" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A28" s="49"/>
       <c r="B28" s="49"/>
-      <c r="C28" s="78" t="s">
+      <c r="C28" s="77" t="s">
         <v>524</v>
       </c>
-      <c r="D28" s="86" t="s">
+      <c r="D28" s="85" t="s">
         <v>561</v>
       </c>
       <c r="F28" s="1"/>
@@ -11452,7 +11501,7 @@
     <row r="29" spans="1:21" s="6" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A29" s="49"/>
       <c r="B29" s="49"/>
-      <c r="C29" s="78" t="s">
+      <c r="C29" s="77" t="s">
         <v>525</v>
       </c>
       <c r="D29" s="49"/>
@@ -11472,10 +11521,10 @@
       <c r="U29" s="21"/>
     </row>
     <row r="30" spans="1:21" s="6" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="81" t="s">
+      <c r="A30" s="80" t="s">
         <v>527</v>
       </c>
-      <c r="B30" s="78" t="s">
+      <c r="B30" s="77" t="s">
         <v>533</v>
       </c>
       <c r="C30" s="49"/>
@@ -11497,10 +11546,10 @@
     </row>
     <row r="31" spans="1:21" s="6" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A31" s="49"/>
-      <c r="B31" s="78" t="s">
+      <c r="B31" s="77" t="s">
         <v>530</v>
       </c>
-      <c r="C31" s="78" t="s">
+      <c r="C31" s="77" t="s">
         <v>529</v>
       </c>
       <c r="D31" s="49"/>
@@ -11520,10 +11569,10 @@
       <c r="U31" s="21"/>
     </row>
     <row r="32" spans="1:21" s="6" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="81" t="s">
+      <c r="A32" s="80" t="s">
         <v>528</v>
       </c>
-      <c r="B32" s="78" t="s">
+      <c r="B32" s="77" t="s">
         <v>532</v>
       </c>
       <c r="C32" s="49"/>
@@ -11545,13 +11594,13 @@
     </row>
     <row r="33" spans="1:21" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A33" s="49"/>
-      <c r="B33" s="78" t="s">
+      <c r="B33" s="77" t="s">
         <v>531</v>
       </c>
-      <c r="C33" s="78" t="s">
+      <c r="C33" s="77" t="s">
         <v>526</v>
       </c>
-      <c r="D33" s="86" t="s">
+      <c r="D33" s="85" t="s">
         <v>562</v>
       </c>
       <c r="F33" s="1"/>
@@ -11592,11 +11641,11 @@
       <c r="U34" s="21"/>
     </row>
     <row r="35" spans="1:21" s="6" customFormat="1" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A35" s="78" t="s">
+      <c r="A35" s="77" t="s">
         <v>539</v>
       </c>
       <c r="B35" s="49"/>
-      <c r="C35" s="78" t="s">
+      <c r="C35" s="77" t="s">
         <v>555</v>
       </c>
       <c r="D35" s="49"/>
@@ -11616,11 +11665,11 @@
       <c r="U35" s="21"/>
     </row>
     <row r="36" spans="1:21" s="6" customFormat="1" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A36" s="78" t="s">
+      <c r="A36" s="77" t="s">
         <v>540</v>
       </c>
       <c r="B36" s="49"/>
-      <c r="C36" s="78" t="s">
+      <c r="C36" s="77" t="s">
         <v>542</v>
       </c>
       <c r="D36" s="49"/>
@@ -11640,11 +11689,11 @@
       <c r="U36" s="21"/>
     </row>
     <row r="37" spans="1:21" s="6" customFormat="1" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A37" s="78" t="s">
+      <c r="A37" s="77" t="s">
         <v>541</v>
       </c>
       <c r="B37" s="49"/>
-      <c r="C37" s="78" t="s">
+      <c r="C37" s="77" t="s">
         <v>556</v>
       </c>
       <c r="D37" s="49"/>
@@ -11686,9 +11735,9 @@
       <c r="U38" s="21"/>
     </row>
     <row r="39" spans="1:21" s="6" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="78"/>
+      <c r="A39" s="77"/>
       <c r="B39" s="49"/>
-      <c r="C39" s="78" t="s">
+      <c r="C39" s="77" t="s">
         <v>546</v>
       </c>
       <c r="D39" s="49"/>
@@ -11708,7 +11757,7 @@
       <c r="U39" s="21"/>
     </row>
     <row r="40" spans="1:21" s="6" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A40" s="83" t="s">
+      <c r="A40" s="82" t="s">
         <v>545</v>
       </c>
       <c r="B40" s="49"/>
@@ -11731,10 +11780,10 @@
     </row>
     <row r="41" spans="1:21" s="6" customFormat="1" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A41" s="49"/>
-      <c r="B41" s="78" t="s">
+      <c r="B41" s="77" t="s">
         <v>548</v>
       </c>
-      <c r="C41" s="78" t="s">
+      <c r="C41" s="77" t="s">
         <v>544</v>
       </c>
       <c r="D41" s="49"/>
@@ -11776,13 +11825,13 @@
       <c r="U42" s="21"/>
     </row>
     <row r="43" spans="1:21" s="6" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A43" s="78" t="s">
+      <c r="A43" s="77" t="s">
         <v>550</v>
       </c>
-      <c r="B43" s="78" t="s">
+      <c r="B43" s="77" t="s">
         <v>554</v>
       </c>
-      <c r="C43" s="78" t="s">
+      <c r="C43" s="77" t="s">
         <v>553</v>
       </c>
       <c r="D43" s="49"/>
@@ -11802,11 +11851,11 @@
       <c r="U43" s="21"/>
     </row>
     <row r="44" spans="1:21" s="6" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="78" t="s">
+      <c r="A44" s="77" t="s">
         <v>551</v>
       </c>
       <c r="B44" s="49"/>
-      <c r="C44" s="78" t="s">
+      <c r="C44" s="77" t="s">
         <v>552</v>
       </c>
       <c r="D44" s="49"/>

</xml_diff>